<commit_message>
removendo o banco de dados
</commit_message>
<xml_diff>
--- a/src/main/resources/customers.xlsx
+++ b/src/main/resources/customers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kelsonthony/Documents/projects/batch-processing/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34AE43F2-FF38-1D45-90D5-2EFAD468F772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BC5FBD-633F-9441-AA2A-51A51DE36F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7340" yWindow="2040" windowWidth="28800" windowHeight="11380" xr2:uid="{EF712562-E35D-480D-985A-DDB7617791B3}"/>
   </bookViews>
@@ -375,15 +375,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -435,15 +440,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54020114-AFD4-41D8-B7AD-9069C986508C}" name="customers" displayName="customers" ref="A1:I16" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I16" xr:uid="{54020114-AFD4-41D8-B7AD-9069C986508C}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{0BF554D3-6CD6-41EE-A194-72EF380408DA}" uniqueName="1" name="id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{06399C04-EFCB-4744-B849-301A3FFE6D00}" uniqueName="2" name="firstName" queryTableFieldId="2" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{717C29CB-C5EE-4AF4-AA28-BA36876B9A73}" uniqueName="3" name="lastName" queryTableFieldId="3" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{3C5CE79F-4D6A-40F7-94D1-F65D79571F3B}" uniqueName="4" name="email" queryTableFieldId="4" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{ECDFE398-6E7A-4417-9420-9FBDDF28F522}" uniqueName="5" name="gender" queryTableFieldId="5" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{566BFE86-DAE7-4895-96B0-DABE2CBAED51}" uniqueName="6" name="contactNo" queryTableFieldId="6" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{FDC0A6BD-D85A-4C2D-93FF-F6755EF35233}" uniqueName="7" name="country" queryTableFieldId="7" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{986E2FE6-A42D-48C3-93A2-9DB5F3C67094}" uniqueName="8" name="dob" queryTableFieldId="8" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{9775E88B-9F78-4882-A0EA-E3AFAE4AAD7D}" uniqueName="9" name="age" queryTableFieldId="9" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{0BF554D3-6CD6-41EE-A194-72EF380408DA}" uniqueName="1" name="id" queryTableFieldId="1" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{06399C04-EFCB-4744-B849-301A3FFE6D00}" uniqueName="2" name="firstName" queryTableFieldId="2" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{717C29CB-C5EE-4AF4-AA28-BA36876B9A73}" uniqueName="3" name="lastName" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{3C5CE79F-4D6A-40F7-94D1-F65D79571F3B}" uniqueName="4" name="email" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{ECDFE398-6E7A-4417-9420-9FBDDF28F522}" uniqueName="5" name="gender" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{566BFE86-DAE7-4895-96B0-DABE2CBAED51}" uniqueName="6" name="contactNo" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{FDC0A6BD-D85A-4C2D-93FF-F6755EF35233}" uniqueName="7" name="country" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{986E2FE6-A42D-48C3-93A2-9DB5F3C67094}" uniqueName="8" name="dob" queryTableFieldId="8" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{9775E88B-9F78-4882-A0EA-E3AFAE4AAD7D}" uniqueName="9" name="age" queryTableFieldId="9" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -810,9 +815,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
+      <c r="A2" s="2"/>
       <c r="B2" t="s">
         <v>9</v>
       </c>
@@ -839,9 +842,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
+      <c r="A3" s="2"/>
       <c r="B3" t="s">
         <v>15</v>
       </c>
@@ -868,9 +869,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
+      <c r="A4" s="2"/>
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -897,9 +896,7 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
+      <c r="A5" s="2"/>
       <c r="B5" t="s">
         <v>29</v>
       </c>
@@ -926,9 +923,7 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
+      <c r="A6" s="2"/>
       <c r="B6" t="s">
         <v>35</v>
       </c>
@@ -955,9 +950,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
+      <c r="A7" s="2"/>
       <c r="B7" t="s">
         <v>41</v>
       </c>
@@ -984,9 +977,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
+      <c r="A8" s="2"/>
       <c r="B8" t="s">
         <v>47</v>
       </c>
@@ -1013,9 +1004,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
+      <c r="A9" s="2"/>
       <c r="B9" t="s">
         <v>53</v>
       </c>
@@ -1042,9 +1031,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" t="s">
         <v>60</v>
       </c>
@@ -1071,9 +1058,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
-      </c>
+      <c r="A11" s="2"/>
       <c r="B11" t="s">
         <v>65</v>
       </c>
@@ -1100,9 +1085,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>11</v>
-      </c>
+      <c r="A12" s="2"/>
       <c r="B12" t="s">
         <v>71</v>
       </c>
@@ -1129,9 +1112,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
-      </c>
+      <c r="A13" s="2"/>
       <c r="B13" t="s">
         <v>75</v>
       </c>
@@ -1158,9 +1139,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>13</v>
-      </c>
+      <c r="A14" s="2"/>
       <c r="B14" t="s">
         <v>79</v>
       </c>
@@ -1187,9 +1166,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>14</v>
-      </c>
+      <c r="A15" s="2"/>
       <c r="B15" t="s">
         <v>84</v>
       </c>
@@ -1216,9 +1193,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
+      <c r="A16" s="2"/>
       <c r="B16" t="s">
         <v>88</v>
       </c>

</xml_diff>